<commit_message>
Refresh RW4 models, outputs, and thesis deliverables
</commit_message>
<xml_diff>
--- a/outputs/run_all_summary/run_all_rw4_summary.xlsx
+++ b/outputs/run_all_summary/run_all_rw4_summary.xlsx
@@ -1362,7 +1362,7 @@
         <v>1</v>
       </c>
       <c r="F13" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -1781,7 +1781,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G111"/>
+  <dimension ref="A1:G118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2244,10 +2244,10 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>279</v>
+        <v>1383</v>
       </c>
       <c r="E16" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F16" t="n">
         <v>1</v>
@@ -2273,7 +2273,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>422</v>
+        <v>1322</v>
       </c>
       <c r="E17" t="n">
         <v>20</v>
@@ -2476,7 +2476,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>422</v>
+        <v>1322</v>
       </c>
       <c r="E24" t="n">
         <v>20</v>
@@ -2505,10 +2505,10 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>7</v>
+        <v>286</v>
       </c>
       <c r="E25" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F25" t="n">
         <v>1</v>
@@ -2853,10 +2853,10 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>722</v>
+        <v>3028</v>
       </c>
       <c r="E37" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F37" t="n">
         <v>1</v>
@@ -2882,16 +2882,16 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E38" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="F38" t="n">
         <v>0</v>
       </c>
       <c r="G38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39">
@@ -2911,10 +2911,10 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>0</v>
+        <v>166</v>
       </c>
       <c r="E39" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F39" t="n">
         <v>0</v>
@@ -2940,10 +2940,10 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>304</v>
+        <v>749</v>
       </c>
       <c r="E40" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F40" t="n">
         <v>1</v>
@@ -2969,10 +2969,10 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>224</v>
+        <v>1992</v>
       </c>
       <c r="E41" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F41" t="n">
         <v>0</v>
@@ -2998,10 +2998,10 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>2574</v>
+        <v>10141</v>
       </c>
       <c r="E42" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F42" t="n">
         <v>1</v>
@@ -3027,10 +3027,10 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>1248</v>
+        <v>4312</v>
       </c>
       <c r="E43" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="F43" t="n">
         <v>1</v>
@@ -3081,14 +3081,14 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>FarmGate_Source_Comparison</t>
+          <t>FarmGate_Direct_Summary</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>654</v>
+        <v>163</v>
       </c>
       <c r="E45" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F45" t="n">
         <v>0</v>
@@ -3110,20 +3110,20 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Mapping_Audit</t>
+          <t>FarmGate_Reverse_Summary</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>3728</v>
+        <v>146</v>
       </c>
       <c r="E46" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="F46" t="n">
         <v>0</v>
       </c>
       <c r="G46" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="47">
@@ -3139,20 +3139,20 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>NARDL_Multipliers</t>
+          <t>FarmGate_Source_Comparison</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>15162</v>
+        <v>2379</v>
       </c>
       <c r="E47" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="F47" t="n">
         <v>0</v>
       </c>
       <c r="G47" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="48">
@@ -3168,14 +3168,14 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Panel_Index</t>
+          <t>FarmGate_Variant_Stability</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>104</v>
+        <v>309</v>
       </c>
       <c r="E48" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F48" t="n">
         <v>0</v>
@@ -3197,20 +3197,20 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>RawMilk_To_Product_Transmission</t>
+          <t>Intersection_Stability</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>253</v>
+        <v>276</v>
       </c>
       <c r="E49" t="n">
-        <v>39</v>
+        <v>10</v>
       </c>
       <c r="F49" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G49" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50">
@@ -3226,14 +3226,14 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Reconstruction_Diagnostics</t>
+          <t>Mapping_Audit</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>55</v>
+        <v>3728</v>
       </c>
       <c r="E50" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F50" t="n">
         <v>0</v>
@@ -3255,20 +3255,20 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Retailer_Brand_Transmission</t>
+          <t>NARDL_Multipliers</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>962</v>
+        <v>63588</v>
       </c>
       <c r="E51" t="n">
-        <v>39</v>
+        <v>8</v>
       </c>
       <c r="F51" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G51" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52">
@@ -3284,20 +3284,20 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>ReverseFlow_ModelCoefficients</t>
+          <t>Panel_Index</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>1137</v>
+        <v>688</v>
       </c>
       <c r="E52" t="n">
-        <v>39</v>
+        <v>16</v>
       </c>
       <c r="F52" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G52" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53">
@@ -3313,20 +3313,20 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Rule_Documentation</t>
+          <t>RawMilk_To_Product_Transmission</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>1</v>
+        <v>3465</v>
       </c>
       <c r="E53" t="n">
-        <v>7</v>
+        <v>41</v>
       </c>
       <c r="F53" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G53" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="54">
@@ -3342,14 +3342,14 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Unit_Admissibility</t>
+          <t>Reconstruction_Diagnostics</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>12</v>
+        <v>55</v>
       </c>
       <c r="E54" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="F54" t="n">
         <v>0</v>
@@ -3371,14 +3371,14 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>VECM_IRF</t>
+          <t>Retail_Combined_Diagnostics</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>2028</v>
+        <v>18</v>
       </c>
       <c r="E55" t="n">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="F55" t="n">
         <v>0</v>
@@ -3400,14 +3400,14 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Variant_Robustness</t>
+          <t>Retail_Combined_Methodology</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>630</v>
+        <v>2</v>
       </c>
       <c r="E56" t="n">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="F56" t="n">
         <v>0</v>
@@ -3419,24 +3419,24 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>model_vecm</t>
+          <t>model_short_chain_regional</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>model_vecm_output.xlsx</t>
+          <t>primary_chain_consolidated.xlsx</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>VECM_Summary</t>
+          <t>Retailer_Brand_Transmission</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>156</v>
+        <v>962</v>
       </c>
       <c r="E57" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F57" t="n">
         <v>1</v>
@@ -3448,53 +3448,53 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>sheet_CME</t>
+          <t>model_short_chain_regional</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>sheet_cme_output.xlsx</t>
+          <t>primary_chain_consolidated.xlsx</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>clean</t>
+          <t>ReverseFlow_ModelCoefficients</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>1023</v>
+        <v>4548</v>
       </c>
       <c r="E58" t="n">
-        <v>27</v>
+        <v>41</v>
       </c>
       <c r="F58" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G58" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>sheet_CME</t>
+          <t>model_short_chain_regional</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>sheet_cme_output.xlsx</t>
+          <t>primary_chain_consolidated.xlsx</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>daily_variants</t>
+          <t>Rule_Documentation</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>1486</v>
+        <v>1</v>
       </c>
       <c r="E59" t="n">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="F59" t="n">
         <v>0</v>
@@ -3506,24 +3506,24 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>sheet_CME</t>
+          <t>model_short_chain_regional</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>sheet_cme_output.xlsx</t>
+          <t>primary_chain_consolidated.xlsx</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>descriptive_stats</t>
+          <t>Unified_Retail_Comparison</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>3</v>
+        <v>212</v>
       </c>
       <c r="E60" t="n">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="F60" t="n">
         <v>0</v>
@@ -3535,24 +3535,24 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>sheet_CME</t>
+          <t>model_short_chain_regional</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>sheet_cme_output.xlsx</t>
+          <t>primary_chain_consolidated.xlsx</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>raw</t>
+          <t>Unit_Admissibility</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>1023</v>
+        <v>12</v>
       </c>
       <c r="E61" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F61" t="n">
         <v>0</v>
@@ -3564,24 +3564,24 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>sheet_CME</t>
+          <t>model_short_chain_regional</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>sheet_cme_output.xlsx</t>
+          <t>primary_chain_consolidated.xlsx</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>series_long</t>
+          <t>VECM_IRF</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>1023</v>
+        <v>3744</v>
       </c>
       <c r="E62" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="F62" t="n">
         <v>0</v>
@@ -3593,82 +3593,82 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>sheet_CME</t>
+          <t>model_short_chain_regional</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>sheet_cme_output.xlsx</t>
+          <t>primary_chain_consolidated.xlsx</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>tests</t>
+          <t>Variant_Robustness</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>3</v>
+        <v>2449</v>
       </c>
       <c r="E63" t="n">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="F63" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G63" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>sheet_ConsumerUA</t>
+          <t>model_vecm</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>sheet_consumerua_output.xlsx</t>
+          <t>model_vecm_output.xlsx</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>clean</t>
+          <t>VECM_Summary</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>5463</v>
+        <v>288</v>
       </c>
       <c r="E64" t="n">
-        <v>30</v>
+        <v>41</v>
       </c>
       <c r="F64" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G64" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>sheet_ConsumerUA</t>
+          <t>sheet_CME</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>sheet_consumerua_output.xlsx</t>
+          <t>sheet_cme_output.xlsx</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>daily_variants</t>
+          <t>clean</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>5463</v>
+        <v>1023</v>
       </c>
       <c r="E65" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F65" t="n">
         <v>0</v>
@@ -3680,24 +3680,24 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>sheet_ConsumerUA</t>
+          <t>sheet_CME</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>sheet_consumerua_output.xlsx</t>
+          <t>sheet_cme_output.xlsx</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>descriptive_stats</t>
+          <t>daily_variants</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>9</v>
+        <v>1486</v>
       </c>
       <c r="E66" t="n">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F66" t="n">
         <v>0</v>
@@ -3709,24 +3709,24 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>sheet_ConsumerUA</t>
+          <t>sheet_CME</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>sheet_consumerua_output.xlsx</t>
+          <t>sheet_cme_output.xlsx</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>raw</t>
+          <t>descriptive_stats</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>5463</v>
+        <v>3</v>
       </c>
       <c r="E67" t="n">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="F67" t="n">
         <v>0</v>
@@ -3738,24 +3738,24 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>sheet_ConsumerUA</t>
+          <t>sheet_CME</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>sheet_consumerua_output.xlsx</t>
+          <t>sheet_cme_output.xlsx</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>series_long</t>
+          <t>raw</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>16389</v>
+        <v>1023</v>
       </c>
       <c r="E68" t="n">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="F68" t="n">
         <v>0</v>
@@ -3767,82 +3767,82 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>sheet_ConsumerUA</t>
+          <t>sheet_CME</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>sheet_consumerua_output.xlsx</t>
+          <t>sheet_cme_output.xlsx</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>tests</t>
+          <t>series_long</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>9</v>
+        <v>1023</v>
       </c>
       <c r="E69" t="n">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="F69" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G69" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>sheet_EU</t>
+          <t>sheet_CME</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>sheet_eu_output.xlsx</t>
+          <t>sheet_cme_output.xlsx</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>clean</t>
+          <t>tests</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>111299</v>
+        <v>3</v>
       </c>
       <c r="E70" t="n">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="F70" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G70" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>sheet_EU</t>
+          <t>sheet_ConsumerUA</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>sheet_eu_output.xlsx</t>
+          <t>sheet_consumerua_output.xlsx</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>daily_variants</t>
+          <t>clean</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>7390</v>
+        <v>5463</v>
       </c>
       <c r="E71" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="F71" t="n">
         <v>0</v>
@@ -3854,24 +3854,24 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>sheet_EU</t>
+          <t>sheet_ConsumerUA</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>sheet_eu_output.xlsx</t>
+          <t>sheet_consumerua_output.xlsx</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>descriptive_stats</t>
+          <t>daily_variants</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>15</v>
+        <v>5463</v>
       </c>
       <c r="E72" t="n">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F72" t="n">
         <v>0</v>
@@ -3883,24 +3883,24 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>sheet_EU</t>
+          <t>sheet_ConsumerUA</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>sheet_eu_output.xlsx</t>
+          <t>sheet_consumerua_output.xlsx</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>raw</t>
+          <t>descriptive_stats</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>111299</v>
+        <v>9</v>
       </c>
       <c r="E73" t="n">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="F73" t="n">
         <v>0</v>
@@ -3912,24 +3912,24 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>sheet_EU</t>
+          <t>sheet_ConsumerUA</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>sheet_eu_output.xlsx</t>
+          <t>sheet_consumerua_output.xlsx</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>series_long</t>
+          <t>raw</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>5280</v>
+        <v>5463</v>
       </c>
       <c r="E74" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="F74" t="n">
         <v>0</v>
@@ -3941,82 +3941,82 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>sheet_EU</t>
+          <t>sheet_ConsumerUA</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>sheet_eu_output.xlsx</t>
+          <t>sheet_consumerua_output.xlsx</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>tests</t>
+          <t>series_long</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>15</v>
+        <v>16389</v>
       </c>
       <c r="E75" t="n">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="F75" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G75" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>sheet_FarmGateUA_filled</t>
+          <t>sheet_ConsumerUA</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>sheet_farmgateua_filled_output.xlsx</t>
+          <t>sheet_consumerua_output.xlsx</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>clean</t>
+          <t>tests</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>38012</v>
+        <v>9</v>
       </c>
       <c r="E76" t="n">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="F76" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G76" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>sheet_FarmGateUA_filled</t>
+          <t>sheet_EU</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>sheet_farmgateua_filled_output.xlsx</t>
+          <t>sheet_eu_output.xlsx</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>daily_variants</t>
+          <t>clean</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>38012</v>
+        <v>111299</v>
       </c>
       <c r="E77" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F77" t="n">
         <v>0</v>
@@ -4028,24 +4028,24 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>sheet_FarmGateUA_filled</t>
+          <t>sheet_EU</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>sheet_farmgateua_filled_output.xlsx</t>
+          <t>sheet_eu_output.xlsx</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>descriptive_stats</t>
+          <t>daily_variants</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>3</v>
+        <v>7390</v>
       </c>
       <c r="E78" t="n">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F78" t="n">
         <v>0</v>
@@ -4057,24 +4057,24 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>sheet_FarmGateUA_filled</t>
+          <t>sheet_EU</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>sheet_farmgateua_filled_output.xlsx</t>
+          <t>sheet_eu_output.xlsx</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>raw</t>
+          <t>descriptive_stats</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>38012</v>
+        <v>15</v>
       </c>
       <c r="E79" t="n">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="F79" t="n">
         <v>0</v>
@@ -4086,24 +4086,24 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>sheet_FarmGateUA_filled</t>
+          <t>sheet_EU</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>sheet_farmgateua_filled_output.xlsx</t>
+          <t>sheet_eu_output.xlsx</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>series_long</t>
+          <t>raw</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>114036</v>
+        <v>111299</v>
       </c>
       <c r="E80" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="F80" t="n">
         <v>0</v>
@@ -4115,82 +4115,82 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>sheet_FarmGateUA_filled</t>
+          <t>sheet_EU</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>sheet_farmgateua_filled_output.xlsx</t>
+          <t>sheet_eu_output.xlsx</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>tests</t>
+          <t>series_long</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>3</v>
+        <v>5280</v>
       </c>
       <c r="E81" t="n">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="F81" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G81" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>sheet_FarmGateUA_initial</t>
+          <t>sheet_EU</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>sheet_farmgateua_initial_output.xlsx</t>
+          <t>sheet_eu_output.xlsx</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>clean</t>
+          <t>tests</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>32620</v>
+        <v>15</v>
       </c>
       <c r="E82" t="n">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="F82" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G82" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>sheet_FarmGateUA_initial</t>
+          <t>sheet_FarmGateUA_filled</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>sheet_farmgateua_initial_output.xlsx</t>
+          <t>sheet_farmgateua_filled_output.xlsx</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>daily_variants</t>
+          <t>clean</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>32620</v>
+        <v>38012</v>
       </c>
       <c r="E83" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="F83" t="n">
         <v>0</v>
@@ -4202,24 +4202,24 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>sheet_FarmGateUA_initial</t>
+          <t>sheet_FarmGateUA_filled</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>sheet_farmgateua_initial_output.xlsx</t>
+          <t>sheet_farmgateua_filled_output.xlsx</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>descriptive_stats</t>
+          <t>daily_variants</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>3</v>
+        <v>38012</v>
       </c>
       <c r="E84" t="n">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F84" t="n">
         <v>0</v>
@@ -4231,24 +4231,24 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>sheet_FarmGateUA_initial</t>
+          <t>sheet_FarmGateUA_filled</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>sheet_farmgateua_initial_output.xlsx</t>
+          <t>sheet_farmgateua_filled_output.xlsx</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>raw</t>
+          <t>descriptive_stats</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>32620</v>
+        <v>3</v>
       </c>
       <c r="E85" t="n">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="F85" t="n">
         <v>0</v>
@@ -4260,24 +4260,24 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>sheet_FarmGateUA_initial</t>
+          <t>sheet_FarmGateUA_filled</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>sheet_farmgateua_initial_output.xlsx</t>
+          <t>sheet_farmgateua_filled_output.xlsx</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>series_long</t>
+          <t>raw</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>97860</v>
+        <v>38012</v>
       </c>
       <c r="E86" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="F86" t="n">
         <v>0</v>
@@ -4289,82 +4289,82 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>sheet_FarmGateUA_initial</t>
+          <t>sheet_FarmGateUA_filled</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>sheet_farmgateua_initial_output.xlsx</t>
+          <t>sheet_farmgateua_filled_output.xlsx</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>tests</t>
+          <t>series_long</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>3</v>
+        <v>114036</v>
       </c>
       <c r="E87" t="n">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="F87" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G87" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>sheet_Novus</t>
+          <t>sheet_FarmGateUA_filled</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>sheet_novus_output.xlsx</t>
+          <t>sheet_farmgateua_filled_output.xlsx</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>clean</t>
+          <t>tests</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>1530</v>
+        <v>3</v>
       </c>
       <c r="E88" t="n">
-        <v>53</v>
+        <v>23</v>
       </c>
       <c r="F88" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G88" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>sheet_Novus</t>
+          <t>sheet_FarmGateUA_initial</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>sheet_novus_output.xlsx</t>
+          <t>sheet_farmgateua_initial_output.xlsx</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>daily_variants</t>
+          <t>clean</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>8654</v>
+        <v>32620</v>
       </c>
       <c r="E89" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="F89" t="n">
         <v>0</v>
@@ -4376,24 +4376,24 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>sheet_Novus</t>
+          <t>sheet_FarmGateUA_initial</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>sheet_novus_output.xlsx</t>
+          <t>sheet_farmgateua_initial_output.xlsx</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>descriptive_stats</t>
+          <t>daily_variants</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>27</v>
+        <v>32620</v>
       </c>
       <c r="E90" t="n">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F90" t="n">
         <v>0</v>
@@ -4405,24 +4405,24 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>sheet_Novus</t>
+          <t>sheet_FarmGateUA_initial</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>sheet_novus_output.xlsx</t>
+          <t>sheet_farmgateua_initial_output.xlsx</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>raw</t>
+          <t>descriptive_stats</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>1530</v>
+        <v>3</v>
       </c>
       <c r="E91" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F91" t="n">
         <v>0</v>
@@ -4434,24 +4434,24 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>sheet_Novus</t>
+          <t>sheet_FarmGateUA_initial</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>sheet_novus_output.xlsx</t>
+          <t>sheet_farmgateua_initial_output.xlsx</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>series_long</t>
+          <t>raw</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>747</v>
+        <v>32620</v>
       </c>
       <c r="E92" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="F92" t="n">
         <v>0</v>
@@ -4463,82 +4463,82 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>sheet_Novus</t>
+          <t>sheet_FarmGateUA_initial</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>sheet_novus_output.xlsx</t>
+          <t>sheet_farmgateua_initial_output.xlsx</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>tests</t>
+          <t>series_long</t>
         </is>
       </c>
       <c r="D93" t="n">
-        <v>27</v>
+        <v>97860</v>
       </c>
       <c r="E93" t="n">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="F93" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G93" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>sheet_ProZorro</t>
+          <t>sheet_FarmGateUA_initial</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>sheet_prozorro_output.xlsx</t>
+          <t>sheet_farmgateua_initial_output.xlsx</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>clean</t>
+          <t>tests</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>10927</v>
+        <v>3</v>
       </c>
       <c r="E94" t="n">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="F94" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G94" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>sheet_ProZorro</t>
+          <t>sheet_Novus</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>sheet_prozorro_output.xlsx</t>
+          <t>sheet_novus_output.xlsx</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>daily_variants</t>
+          <t>clean</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>35275</v>
+        <v>1530</v>
       </c>
       <c r="E95" t="n">
-        <v>25</v>
+        <v>53</v>
       </c>
       <c r="F95" t="n">
         <v>0</v>
@@ -4550,24 +4550,24 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>sheet_ProZorro</t>
+          <t>sheet_Novus</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>sheet_prozorro_output.xlsx</t>
+          <t>sheet_novus_output.xlsx</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>descriptive_stats</t>
+          <t>daily_variants</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>18</v>
+        <v>8654</v>
       </c>
       <c r="E96" t="n">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F96" t="n">
         <v>0</v>
@@ -4579,24 +4579,24 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>sheet_ProZorro</t>
+          <t>sheet_Novus</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>sheet_prozorro_output.xlsx</t>
+          <t>sheet_novus_output.xlsx</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>raw</t>
+          <t>descriptive_stats</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>10927</v>
+        <v>27</v>
       </c>
       <c r="E97" t="n">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="F97" t="n">
         <v>0</v>
@@ -4608,24 +4608,24 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>sheet_ProZorro</t>
+          <t>sheet_Novus</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>sheet_prozorro_output.xlsx</t>
+          <t>sheet_novus_output.xlsx</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>series_long</t>
+          <t>raw</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>7239</v>
+        <v>1530</v>
       </c>
       <c r="E98" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="F98" t="n">
         <v>0</v>
@@ -4637,82 +4637,82 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>sheet_ProZorro</t>
+          <t>sheet_Novus</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>sheet_prozorro_output.xlsx</t>
+          <t>sheet_novus_output.xlsx</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>tests</t>
+          <t>series_long</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>18</v>
+        <v>747</v>
       </c>
       <c r="E99" t="n">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="F99" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G99" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>sheet_ProducerUA</t>
+          <t>sheet_Novus</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>sheet_producerua_output.xlsx</t>
+          <t>sheet_novus_output.xlsx</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>clean</t>
+          <t>tests</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>10758</v>
+        <v>27</v>
       </c>
       <c r="E100" t="n">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="F100" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G100" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>sheet_ProducerUA</t>
+          <t>sheet_ProZorro</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>sheet_producerua_output.xlsx</t>
+          <t>sheet_prozorro_output.xlsx</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>daily_variants</t>
+          <t>clean</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>8965</v>
+        <v>10927</v>
       </c>
       <c r="E101" t="n">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="F101" t="n">
         <v>0</v>
@@ -4724,24 +4724,24 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>sheet_ProducerUA</t>
+          <t>sheet_ProZorro</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>sheet_producerua_output.xlsx</t>
+          <t>sheet_prozorro_output.xlsx</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>descriptive_stats</t>
+          <t>daily_variants</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>15</v>
+        <v>35275</v>
       </c>
       <c r="E102" t="n">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F102" t="n">
         <v>0</v>
@@ -4753,24 +4753,24 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>sheet_ProducerUA</t>
+          <t>sheet_ProZorro</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>sheet_producerua_output.xlsx</t>
+          <t>sheet_prozorro_output.xlsx</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>raw</t>
+          <t>descriptive_stats</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>10758</v>
+        <v>18</v>
       </c>
       <c r="E103" t="n">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="F103" t="n">
         <v>0</v>
@@ -4782,24 +4782,24 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>sheet_ProducerUA</t>
+          <t>sheet_ProZorro</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>sheet_producerua_output.xlsx</t>
+          <t>sheet_prozorro_output.xlsx</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>series_long</t>
+          <t>raw</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>26895</v>
+        <v>10927</v>
       </c>
       <c r="E104" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F104" t="n">
         <v>0</v>
@@ -4811,82 +4811,82 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>sheet_ProducerUA</t>
+          <t>sheet_ProZorro</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>sheet_producerua_output.xlsx</t>
+          <t>sheet_prozorro_output.xlsx</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>tests</t>
+          <t>series_long</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>15</v>
+        <v>7239</v>
       </c>
       <c r="E105" t="n">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="F105" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G105" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>sheet_Silpo</t>
+          <t>sheet_ProZorro</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>sheet_silpo_output.xlsx</t>
+          <t>sheet_prozorro_output.xlsx</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>clean</t>
+          <t>tests</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>86765</v>
+        <v>18</v>
       </c>
       <c r="E106" t="n">
-        <v>53</v>
+        <v>23</v>
       </c>
       <c r="F106" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G106" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>sheet_Silpo</t>
+          <t>sheet_ProducerUA</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>sheet_silpo_output.xlsx</t>
+          <t>sheet_producerua_output.xlsx</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>daily_variants</t>
+          <t>clean</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>22120</v>
+        <v>10758</v>
       </c>
       <c r="E107" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="F107" t="n">
         <v>0</v>
@@ -4898,24 +4898,24 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>sheet_Silpo</t>
+          <t>sheet_ProducerUA</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>sheet_silpo_output.xlsx</t>
+          <t>sheet_producerua_output.xlsx</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>descriptive_stats</t>
+          <t>daily_variants</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>24</v>
+        <v>8965</v>
       </c>
       <c r="E108" t="n">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F108" t="n">
         <v>0</v>
@@ -4927,24 +4927,24 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>sheet_Silpo</t>
+          <t>sheet_ProducerUA</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>sheet_silpo_output.xlsx</t>
+          <t>sheet_producerua_output.xlsx</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>raw</t>
+          <t>descriptive_stats</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>86765</v>
+        <v>15</v>
       </c>
       <c r="E109" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F109" t="n">
         <v>0</v>
@@ -4956,24 +4956,24 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>sheet_Silpo</t>
+          <t>sheet_ProducerUA</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>sheet_silpo_output.xlsx</t>
+          <t>sheet_producerua_output.xlsx</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>series_long</t>
+          <t>raw</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>19508</v>
+        <v>10758</v>
       </c>
       <c r="E110" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="F110" t="n">
         <v>0</v>
@@ -4985,29 +4985,232 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
+          <t>sheet_ProducerUA</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>sheet_producerua_output.xlsx</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>series_long</t>
+        </is>
+      </c>
+      <c r="D111" t="n">
+        <v>26895</v>
+      </c>
+      <c r="E111" t="n">
+        <v>16</v>
+      </c>
+      <c r="F111" t="n">
+        <v>0</v>
+      </c>
+      <c r="G111" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>sheet_ProducerUA</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>sheet_producerua_output.xlsx</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>tests</t>
+        </is>
+      </c>
+      <c r="D112" t="n">
+        <v>15</v>
+      </c>
+      <c r="E112" t="n">
+        <v>23</v>
+      </c>
+      <c r="F112" t="n">
+        <v>1</v>
+      </c>
+      <c r="G112" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
           <t>sheet_Silpo</t>
         </is>
       </c>
-      <c r="B111" t="inlineStr">
+      <c r="B113" t="inlineStr">
         <is>
           <t>sheet_silpo_output.xlsx</t>
         </is>
       </c>
-      <c r="C111" t="inlineStr">
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>clean</t>
+        </is>
+      </c>
+      <c r="D113" t="n">
+        <v>86765</v>
+      </c>
+      <c r="E113" t="n">
+        <v>53</v>
+      </c>
+      <c r="F113" t="n">
+        <v>0</v>
+      </c>
+      <c r="G113" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>sheet_Silpo</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>sheet_silpo_output.xlsx</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>daily_variants</t>
+        </is>
+      </c>
+      <c r="D114" t="n">
+        <v>22120</v>
+      </c>
+      <c r="E114" t="n">
+        <v>25</v>
+      </c>
+      <c r="F114" t="n">
+        <v>0</v>
+      </c>
+      <c r="G114" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>sheet_Silpo</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>sheet_silpo_output.xlsx</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>descriptive_stats</t>
+        </is>
+      </c>
+      <c r="D115" t="n">
+        <v>24</v>
+      </c>
+      <c r="E115" t="n">
+        <v>21</v>
+      </c>
+      <c r="F115" t="n">
+        <v>0</v>
+      </c>
+      <c r="G115" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>sheet_Silpo</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>sheet_silpo_output.xlsx</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="D116" t="n">
+        <v>86765</v>
+      </c>
+      <c r="E116" t="n">
+        <v>19</v>
+      </c>
+      <c r="F116" t="n">
+        <v>0</v>
+      </c>
+      <c r="G116" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>sheet_Silpo</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>sheet_silpo_output.xlsx</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>series_long</t>
+        </is>
+      </c>
+      <c r="D117" t="n">
+        <v>19508</v>
+      </c>
+      <c r="E117" t="n">
+        <v>16</v>
+      </c>
+      <c r="F117" t="n">
+        <v>0</v>
+      </c>
+      <c r="G117" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>sheet_Silpo</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>sheet_silpo_output.xlsx</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
         <is>
           <t>tests</t>
         </is>
       </c>
-      <c r="D111" t="n">
+      <c r="D118" t="n">
         <v>24</v>
       </c>
-      <c r="E111" t="n">
+      <c r="E118" t="n">
         <v>23</v>
       </c>
-      <c r="F111" t="n">
-        <v>1</v>
-      </c>
-      <c r="G111" t="n">
+      <c r="F118" t="n">
+        <v>1</v>
+      </c>
+      <c r="G118" t="n">
         <v>1</v>
       </c>
     </row>
@@ -5079,7 +5282,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>279</v>
+        <v>1383</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
@@ -5110,7 +5313,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>7</v>
+        <v>286</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
@@ -5141,7 +5344,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>722</v>
+        <v>3028</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
@@ -5172,7 +5375,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>304</v>
+        <v>749</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
@@ -5203,7 +5406,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2574</v>
+        <v>10141</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
@@ -5234,17 +5437,17 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1248</v>
+        <v>4312</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>0.3966346153846154</v>
+        <v>0.5051020408163265</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>I(1)-like share=0.00; cointegration-support share=0.40; inspect admissibility and reconstruction robustness before promoting findings.</t>
+          <t>I(1)-like share=0.00; cointegration-support share=0.51; inspect admissibility and reconstruction robustness before promoting findings.</t>
         </is>
       </c>
     </row>
@@ -5265,7 +5468,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>253</v>
+        <v>3465</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
@@ -5327,7 +5530,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>1137</v>
+        <v>4548</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
@@ -5358,7 +5561,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>156</v>
+        <v>288</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
@@ -5662,7 +5865,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5746,7 +5949,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>279</v>
+        <v>1383</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
@@ -5756,7 +5959,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>mean |coef|=2.8478 | significance share (p&lt;0.05)=0.13 | robust-across-reconstruction share=0.00 | core-finding share=0.00</t>
+          <t>mean |coef|=2.6492 | significance share (p&lt;0.05)=0.33 | robust-across-reconstruction share=0.00 | core-finding share=0.00</t>
         </is>
       </c>
     </row>
@@ -5777,13 +5980,13 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>422</v>
+        <v>1322</v>
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>mean |coef|=4.8410</t>
+          <t>mean |coef|=3.4146</t>
         </is>
       </c>
     </row>
@@ -5804,13 +6007,13 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>422</v>
+        <v>1322</v>
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>mean |coef|=4.8410</t>
+          <t>mean |coef|=3.4146</t>
         </is>
       </c>
     </row>
@@ -5831,17 +6034,17 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>7</v>
+        <v>286</v>
       </c>
       <c r="E6" t="n">
-        <v>0.5714285714285714</v>
+        <v>0.8951048951048951</v>
       </c>
       <c r="F6" t="n">
-        <v>0.5714285714285714</v>
+        <v>0.1013986013986014</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>mean |coef|=0.7894 | significance share (p&lt;0.05)=0.29 | robust-across-reconstruction share=0.57 | core-finding share=0.57</t>
+          <t>mean |coef|=0.7494 | significance share (p&lt;0.05)=0.74 | robust-across-reconstruction share=0.90 | core-finding share=0.10</t>
         </is>
       </c>
     </row>
@@ -5916,48 +6119,44 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>722</v>
+        <v>3028</v>
       </c>
       <c r="E9" t="n">
-        <v>0.7036011080332411</v>
+        <v>0.8127476882430648</v>
       </c>
       <c r="F9" t="n">
-        <v>0.3781163434903047</v>
+        <v>0.2807133421400264</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>mean |coef|=8.3676 | significance share (p&lt;0.05)=0.31 | robust-across-reconstruction share=0.70 | core-finding share=0.38</t>
+          <t>mean |coef|=4.1309 | significance share (p&lt;0.05)=0.43 | robust-across-reconstruction share=0.81 | core-finding share=0.28</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>model_short_chain_regional</t>
+          <t>model_secondary_synthetic_consumer</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>primary_chain_consolidated.xlsx</t>
+          <t>secondary_synthetic_consumer_output.xlsx</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>AveragePrice_Chain_Transmission</t>
+          <t>Synthetic_Consumer_Link</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>304</v>
-      </c>
-      <c r="E10" t="n">
-        <v>0.3092105263157895</v>
-      </c>
-      <c r="F10" t="n">
-        <v>0.1151315789473684</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>mean |coef|=4.5816 | significance share (p&lt;0.05)=0.37 | robust-across-reconstruction share=0.31 | core-finding share=0.12</t>
+          <t>mean |coef|=0.4950 | significance share (p&lt;0.05)=0.50</t>
         </is>
       </c>
     </row>
@@ -5974,21 +6173,21 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Consolidated_ModelCoefficients</t>
+          <t>AveragePrice_Chain_Transmission</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>2574</v>
+        <v>749</v>
       </c>
       <c r="E11" t="n">
-        <v>0.1989121989121989</v>
+        <v>0.2590120160213618</v>
       </c>
       <c r="F11" t="n">
-        <v>0.1076146076146076</v>
+        <v>0.1121495327102804</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>mean |coef|=7.4847 | significance share (p&lt;0.05)=0.26 | robust-across-reconstruction share=0.20 | core-finding share=0.11</t>
+          <t>mean |coef|=2.9094 | significance share (p&lt;0.05)=0.31 | robust-across-reconstruction share=0.26 | core-finding share=0.11</t>
         </is>
       </c>
     </row>
@@ -6005,17 +6204,21 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Consolidated_PreTests</t>
+          <t>Consolidated_ModelCoefficients</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>1248</v>
-      </c>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
+        <v>10141</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.2679222956315945</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.08667784242185189</v>
+      </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>significance share (p&lt;0.05)=0.45</t>
+          <t>mean |coef|=3.5293 | significance share (p&lt;0.05)=0.41 | robust-across-reconstruction share=0.27 | core-finding share=0.09</t>
         </is>
       </c>
     </row>
@@ -6032,19 +6235,17 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>FarmGate_Source_Comparison</t>
+          <t>Consolidated_PreTests</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>654</v>
-      </c>
-      <c r="E13" t="n">
-        <v>0.3914373088685015</v>
-      </c>
+        <v>4312</v>
+      </c>
+      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>robust-across-reconstruction share=0.39</t>
+          <t>significance share (p&lt;0.05)=0.49</t>
         </is>
       </c>
     </row>
@@ -6061,21 +6262,17 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>RawMilk_To_Product_Transmission</t>
+          <t>FarmGate_Direct_Summary</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>253</v>
-      </c>
-      <c r="E14" t="n">
-        <v>0.1422924901185771</v>
-      </c>
-      <c r="F14" t="n">
-        <v>0.003952569169960474</v>
-      </c>
+        <v>163</v>
+      </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>mean |coef|=8.5131 | significance share (p&lt;0.05)=0.20 | robust-across-reconstruction share=0.14 | core-finding share=0.00</t>
+          <t>mean |coef|=8.5959</t>
         </is>
       </c>
     </row>
@@ -6092,21 +6289,17 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Retailer_Brand_Transmission</t>
+          <t>FarmGate_Reverse_Summary</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>962</v>
-      </c>
-      <c r="E15" t="n">
-        <v>0.1268191268191268</v>
-      </c>
-      <c r="F15" t="n">
-        <v>0.05717255717255718</v>
-      </c>
+        <v>146</v>
+      </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>mean |coef|=8.4973 | significance share (p&lt;0.05)=0.27 | robust-across-reconstruction share=0.13 | core-finding share=0.06</t>
+          <t>mean |coef|=0.1189</t>
         </is>
       </c>
     </row>
@@ -6123,145 +6316,155 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>ReverseFlow_ModelCoefficients</t>
+          <t>FarmGate_Source_Comparison</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>1137</v>
+        <v>2379</v>
       </c>
       <c r="E16" t="n">
-        <v>0.2269129287598945</v>
-      </c>
-      <c r="F16" t="n">
-        <v>0.1266490765171504</v>
-      </c>
+        <v>0.4888608659100462</v>
+      </c>
+      <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>mean |coef|=0.4251 | significance share (p&lt;0.05)=0.33 | robust-across-reconstruction share=0.23 | core-finding share=0.13</t>
+          <t>robust-across-reconstruction share=0.49</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>model_vecm</t>
+          <t>model_short_chain_regional</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>model_vecm_output.xlsx</t>
+          <t>primary_chain_consolidated.xlsx</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>VECM_Summary</t>
+          <t>RawMilk_To_Product_Transmission</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>156</v>
+        <v>3465</v>
       </c>
       <c r="E17" t="n">
-        <v>0</v>
+        <v>0.236940836940837</v>
       </c>
       <c r="F17" t="n">
-        <v>0</v>
+        <v>0.02655122655122655</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>mean |coef|=21.7232 | significance share (p&lt;0.05)=0.09 | robust-across-reconstruction share=0.00 | core-finding share=0.00</t>
+          <t>mean |coef|=8.1330 | significance share (p&lt;0.05)=0.39 | robust-across-reconstruction share=0.24 | core-finding share=0.03</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>sheet_CME</t>
+          <t>model_short_chain_regional</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>sheet_cme_output.xlsx</t>
+          <t>primary_chain_consolidated.xlsx</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>tests</t>
+          <t>Retailer_Brand_Transmission</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>3</v>
-      </c>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
+        <v>962</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0.1268191268191268</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0.05717255717255718</v>
+      </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>significance share (p&lt;0.05)=0.50</t>
+          <t>mean |coef|=8.4973 | significance share (p&lt;0.05)=0.27 | robust-across-reconstruction share=0.13 | core-finding share=0.06</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>sheet_ConsumerUA</t>
+          <t>model_short_chain_regional</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>sheet_consumerua_output.xlsx</t>
+          <t>primary_chain_consolidated.xlsx</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>tests</t>
+          <t>ReverseFlow_ModelCoefficients</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>9</v>
-      </c>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
+        <v>4548</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0.2897977132805629</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.1018029903254178</v>
+      </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>significance share (p&lt;0.05)=0.67</t>
+          <t>mean |coef|=0.3376 | significance share (p&lt;0.05)=0.44 | robust-across-reconstruction share=0.29 | core-finding share=0.10</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>sheet_EU</t>
+          <t>model_vecm</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>sheet_eu_output.xlsx</t>
+          <t>model_vecm_output.xlsx</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>tests</t>
+          <t>VECM_Summary</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>15</v>
-      </c>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
+        <v>288</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0</v>
+      </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>significance share (p&lt;0.05)=0.50</t>
+          <t>mean |coef|=11.6733 | significance share (p&lt;0.05)=0.23 | robust-across-reconstruction share=0.00 | core-finding share=0.00</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>sheet_FarmGateUA_filled</t>
+          <t>sheet_CME</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>sheet_farmgateua_filled_output.xlsx</t>
+          <t>sheet_cme_output.xlsx</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -6276,19 +6479,19 @@
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>significance share (p&lt;0.05)=0.67</t>
+          <t>significance share (p&lt;0.05)=0.50</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>sheet_FarmGateUA_initial</t>
+          <t>sheet_ConsumerUA</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>sheet_farmgateua_initial_output.xlsx</t>
+          <t>sheet_consumerua_output.xlsx</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -6297,25 +6500,25 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
-          <t>significance share (p&lt;0.05)=0.83</t>
+          <t>significance share (p&lt;0.05)=0.67</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>sheet_Novus</t>
+          <t>sheet_EU</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>sheet_novus_output.xlsx</t>
+          <t>sheet_eu_output.xlsx</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -6324,25 +6527,25 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Result table has no standard coefficient/p-value columns; interpret by table-specific fields.</t>
+          <t>significance share (p&lt;0.05)=0.50</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>sheet_ProZorro</t>
+          <t>sheet_FarmGateUA_filled</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>sheet_prozorro_output.xlsx</t>
+          <t>sheet_farmgateua_filled_output.xlsx</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -6351,25 +6554,25 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
-          <t>significance share (p&lt;0.05)=0.25</t>
+          <t>significance share (p&lt;0.05)=0.67</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>sheet_ProducerUA</t>
+          <t>sheet_FarmGateUA_initial</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>sheet_producerua_output.xlsx</t>
+          <t>sheet_farmgateua_initial_output.xlsx</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -6378,25 +6581,25 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
-          <t>significance share (p&lt;0.05)=0.67</t>
+          <t>significance share (p&lt;0.05)=0.83</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>sheet_Silpo</t>
+          <t>sheet_Novus</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>sheet_silpo_output.xlsx</t>
+          <t>sheet_novus_output.xlsx</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -6405,11 +6608,92 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
+        <is>
+          <t>Result table has no standard coefficient/p-value columns; interpret by table-specific fields.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>sheet_ProZorro</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>sheet_prozorro_output.xlsx</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>tests</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>18</v>
+      </c>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>significance share (p&lt;0.05)=0.25</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>sheet_ProducerUA</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>sheet_producerua_output.xlsx</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>tests</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>15</v>
+      </c>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>significance share (p&lt;0.05)=0.67</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>sheet_Silpo</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>sheet_silpo_output.xlsx</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>tests</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>24</v>
+      </c>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr">
         <is>
           <t>Result table has no standard coefficient/p-value columns; interpret by table-specific fields.</t>
         </is>
@@ -6637,7 +6921,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>I(1)-like share=0.00; cointegration-support share=0.00; inspect admissibility and reconstruction robustness before promoting findings. | mean |coef|=2.8478 | significance share (p&lt;0.05)=0.13 | robust-across-reconstruction share=0.00 | core-finding share=0.00</t>
+          <t>I(1)-like share=0.00; cointegration-support share=0.00; inspect admissibility and reconstruction robustness before promoting findings. | mean |coef|=2.6492 | significance share (p&lt;0.05)=0.33 | robust-across-reconstruction share=0.00 | core-finding share=0.00</t>
         </is>
       </c>
     </row>
@@ -6672,7 +6956,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>mean |coef|=4.8410</t>
+          <t>mean |coef|=3.4146</t>
         </is>
       </c>
     </row>
@@ -6707,7 +6991,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>I(1)-like share=0.00; cointegration-support share=0.00; inspect admissibility and reconstruction robustness before promoting findings. | mean |coef|=0.7894 | significance share (p&lt;0.05)=0.29 | robust-across-reconstruction share=0.57 | core-finding share=0.57</t>
+          <t>I(1)-like share=0.00; cointegration-support share=0.00; inspect admissibility and reconstruction robustness before promoting findings. | mean |coef|=0.7494 | significance share (p&lt;0.05)=0.74 | robust-across-reconstruction share=0.90 | core-finding share=0.10</t>
         </is>
       </c>
     </row>
@@ -6812,7 +7096,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>I(1)-like share=0.00; cointegration-support share=0.00; inspect admissibility and reconstruction robustness before promoting findings. | mean |coef|=8.3676 | significance share (p&lt;0.05)=0.31 | robust-across-reconstruction share=0.70 | core-finding share=0.38</t>
+          <t>I(1)-like share=0.00; cointegration-support share=0.00; inspect admissibility and reconstruction robustness before promoting findings. | mean |coef|=4.1309 | significance share (p&lt;0.05)=0.43 | robust-across-reconstruction share=0.81 | core-finding share=0.28</t>
         </is>
       </c>
     </row>
@@ -6847,7 +7131,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>No explicit test/model tables detected; inspect module-specific outputs.</t>
+          <t>mean |coef|=0.4950 | significance share (p&lt;0.05)=0.50</t>
         </is>
       </c>
     </row>
@@ -6878,11 +7162,11 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>I(1)-like share=0.00; cointegration-support share=0.00; inspect admissibility and reconstruction robustness before promoting findings. | mean |coef|=7.4847 | significance share (p&lt;0.05)=0.26 | robust-across-reconstruction share=0.20 | core-finding share=0.11</t>
+          <t>I(1)-like share=0.00; cointegration-support share=0.00; inspect admissibility and reconstruction robustness before promoting findings. | mean |coef|=3.5293 | significance share (p&lt;0.05)=0.41 | robust-across-reconstruction share=0.27 | core-finding share=0.09</t>
         </is>
       </c>
     </row>
@@ -6917,7 +7201,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>I(1)-like share=0.00; cointegration-support share=0.00; inspect admissibility and reconstruction robustness before promoting findings. | mean |coef|=21.7232 | significance share (p&lt;0.05)=0.09 | robust-across-reconstruction share=0.00 | core-finding share=0.00</t>
+          <t>I(1)-like share=0.00; cointegration-support share=0.00; inspect admissibility and reconstruction robustness before promoting findings. | mean |coef|=11.6733 | significance share (p&lt;0.05)=0.23 | robust-across-reconstruction share=0.00 | core-finding share=0.00</t>
         </is>
       </c>
     </row>

</xml_diff>